<commit_message>
add a new site to the canopy pre-fit examples and keep Macrocystis-only sites in the Macrocystis one
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-raw/workbooks/kelpbio-4-canopy-prefit-macro.xlsx
+++ b/data-raw/workbooks/kelpbio-4-canopy-prefit-macro.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>site</t>
   </si>
@@ -34,9 +34,6 @@
     <t>Golden</t>
   </si>
   <si>
-    <t>Manley</t>
-  </si>
-  <si>
     <t>Meay</t>
   </si>
   <si>
@@ -49,13 +46,13 @@
     <t>Triquet</t>
   </si>
   <si>
-    <t>Triquetta</t>
-  </si>
-  <si>
     <t>Westbeach</t>
   </si>
   <si>
     <t>Womanley</t>
+  </si>
+  <si>
+    <t>New site</t>
   </si>
 </sst>
 </file>
@@ -398,7 +395,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1">
@@ -443,13 +440,13 @@
         <v>2026</v>
       </c>
       <c r="C3">
-        <v>7552</v>
+        <v>9210</v>
       </c>
       <c r="D3">
-        <v>1.6</v>
+        <v>0.65</v>
       </c>
       <c r="E3">
-        <v>15993</v>
+        <v>21098</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -460,13 +457,13 @@
         <v>2026</v>
       </c>
       <c r="C4">
-        <v>9210</v>
+        <v>7102</v>
       </c>
       <c r="D4">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="E4">
-        <v>21098</v>
+        <v>18281</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -477,13 +474,13 @@
         <v>2026</v>
       </c>
       <c r="C5">
-        <v>7102</v>
+        <v>4769</v>
       </c>
       <c r="D5">
-        <v>0.75</v>
+        <v>0.55</v>
       </c>
       <c r="E5">
-        <v>18281</v>
+        <v>10539</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -494,13 +491,13 @@
         <v>2026</v>
       </c>
       <c r="C6">
-        <v>4769</v>
+        <v>5473</v>
       </c>
       <c r="D6">
-        <v>0.55</v>
+        <v>0.75</v>
       </c>
       <c r="E6">
-        <v>10539</v>
+        <v>9263</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -511,13 +508,13 @@
         <v>2026</v>
       </c>
       <c r="C7">
-        <v>5473</v>
+        <v>7367</v>
       </c>
       <c r="D7">
-        <v>0.75</v>
+        <v>0.1</v>
       </c>
       <c r="E7">
-        <v>9263</v>
+        <v>16615</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -528,13 +525,13 @@
         <v>2026</v>
       </c>
       <c r="C8">
-        <v>659</v>
+        <v>3611</v>
       </c>
       <c r="D8">
-        <v>0.1</v>
+        <v>1.25</v>
       </c>
       <c r="E8">
-        <v>1443</v>
+        <v>9036</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -545,30 +542,13 @@
         <v>2026</v>
       </c>
       <c r="C9">
-        <v>7367</v>
+        <v>8801</v>
       </c>
       <c r="D9">
-        <v>0.1</v>
+        <v>1.25</v>
       </c>
       <c r="E9">
-        <v>16615</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10">
-        <v>2026</v>
-      </c>
-      <c r="C10">
-        <v>3611</v>
-      </c>
-      <c r="D10">
-        <v>1.25</v>
-      </c>
-      <c r="E10">
-        <v>9036</v>
+        <v>24287</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
leave Golden and Womanley out of the Macrocystis canopy pre-fit example
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-raw/workbooks/kelpbio-4-canopy-prefit-macro.xlsx
+++ b/data-raw/workbooks/kelpbio-4-canopy-prefit-macro.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>site</t>
   </si>
@@ -31,9 +31,6 @@
     <t>classified_area_m2</t>
   </si>
   <si>
-    <t>Golden</t>
-  </si>
-  <si>
     <t>Meay</t>
   </si>
   <si>
@@ -47,9 +44,6 @@
   </si>
   <si>
     <t>Westbeach</t>
-  </si>
-  <si>
-    <t>Womanley</t>
   </si>
   <si>
     <t>New site</t>
@@ -395,7 +389,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1">
@@ -423,13 +417,13 @@
         <v>2026</v>
       </c>
       <c r="C2">
-        <v>8801</v>
+        <v>9210</v>
       </c>
       <c r="D2">
-        <v>1.25</v>
+        <v>0.65</v>
       </c>
       <c r="E2">
-        <v>24287</v>
+        <v>21098</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -440,13 +434,13 @@
         <v>2026</v>
       </c>
       <c r="C3">
-        <v>9210</v>
+        <v>7102</v>
       </c>
       <c r="D3">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="E3">
-        <v>21098</v>
+        <v>18281</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -457,13 +451,13 @@
         <v>2026</v>
       </c>
       <c r="C4">
-        <v>7102</v>
+        <v>4769</v>
       </c>
       <c r="D4">
-        <v>0.75</v>
+        <v>0.55</v>
       </c>
       <c r="E4">
-        <v>18281</v>
+        <v>10539</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -474,13 +468,13 @@
         <v>2026</v>
       </c>
       <c r="C5">
-        <v>4769</v>
+        <v>5473</v>
       </c>
       <c r="D5">
-        <v>0.55</v>
+        <v>0.75</v>
       </c>
       <c r="E5">
-        <v>10539</v>
+        <v>9263</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -491,13 +485,13 @@
         <v>2026</v>
       </c>
       <c r="C6">
-        <v>5473</v>
+        <v>7367</v>
       </c>
       <c r="D6">
-        <v>0.75</v>
+        <v>0.1</v>
       </c>
       <c r="E6">
-        <v>9263</v>
+        <v>16615</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -508,47 +502,13 @@
         <v>2026</v>
       </c>
       <c r="C7">
-        <v>7367</v>
+        <v>9210</v>
       </c>
       <c r="D7">
-        <v>0.1</v>
+        <v>0.65</v>
       </c>
       <c r="E7">
-        <v>16615</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8">
-        <v>2026</v>
-      </c>
-      <c r="C8">
-        <v>3611</v>
-      </c>
-      <c r="D8">
-        <v>1.25</v>
-      </c>
-      <c r="E8">
-        <v>9036</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9">
-        <v>2026</v>
-      </c>
-      <c r="C9">
-        <v>8801</v>
-      </c>
-      <c r="D9">
-        <v>1.25</v>
-      </c>
-      <c r="E9">
-        <v>24287</v>
+        <v>21098</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
rebuild the example workbooks from kelpbio's current simulated data, which converge at the default sampler settings
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-raw/workbooks/kelpbio-4-canopy-prefit-macro.xlsx
+++ b/data-raw/workbooks/kelpbio-4-canopy-prefit-macro.xlsx
@@ -417,13 +417,13 @@
         <v>2026</v>
       </c>
       <c r="C2">
-        <v>9210</v>
+        <v>11785</v>
       </c>
       <c r="D2">
-        <v>0.65</v>
+        <v>0.1</v>
       </c>
       <c r="E2">
-        <v>21098</v>
+        <v>23032</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -434,13 +434,13 @@
         <v>2026</v>
       </c>
       <c r="C3">
-        <v>7102</v>
+        <v>2504</v>
       </c>
       <c r="D3">
-        <v>0.75</v>
+        <v>0.35</v>
       </c>
       <c r="E3">
-        <v>18281</v>
+        <v>5272</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -451,13 +451,13 @@
         <v>2026</v>
       </c>
       <c r="C4">
-        <v>4769</v>
+        <v>8071</v>
       </c>
       <c r="D4">
-        <v>0.55</v>
+        <v>0.5</v>
       </c>
       <c r="E4">
-        <v>10539</v>
+        <v>17723</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -468,13 +468,13 @@
         <v>2026</v>
       </c>
       <c r="C5">
-        <v>5473</v>
+        <v>5719</v>
       </c>
       <c r="D5">
-        <v>0.75</v>
+        <v>1.55</v>
       </c>
       <c r="E5">
-        <v>9263</v>
+        <v>14871</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -485,13 +485,13 @@
         <v>2026</v>
       </c>
       <c r="C6">
-        <v>7367</v>
+        <v>7459</v>
       </c>
       <c r="D6">
-        <v>0.1</v>
+        <v>1.45</v>
       </c>
       <c r="E6">
-        <v>16615</v>
+        <v>15578</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -502,13 +502,13 @@
         <v>2026</v>
       </c>
       <c r="C7">
-        <v>9210</v>
+        <v>11785</v>
       </c>
       <c r="D7">
-        <v>0.65</v>
+        <v>0.1</v>
       </c>
       <c r="E7">
-        <v>21098</v>
+        <v>23032</v>
       </c>
     </row>
   </sheetData>

</xml_diff>